<commit_message>
changing Array to Microarray
</commit_message>
<xml_diff>
--- a/inst/extdata/Curated_datasets.xlsx
+++ b/inst/extdata/Curated_datasets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahmedsalah/DoReMiTra/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F29F969D-9100-7F4A-A864-342A54E96556}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C0DFC73-85D1-8247-9D80-0A9A530888DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20320" xr2:uid="{70D3F6C7-018C-1D43-8B93-4E2D6206F13E}"/>
   </bookViews>
@@ -95,9 +95,6 @@
     <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE124612</t>
   </si>
   <si>
-    <t>Array</t>
-  </si>
-  <si>
     <t>Healthy</t>
   </si>
   <si>
@@ -736,6 +733,9 @@
   </si>
   <si>
     <t>GitHub</t>
+  </si>
+  <si>
+    <t>Microarray</t>
   </si>
 </sst>
 </file>
@@ -1202,7 +1202,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -1211,7 +1211,7 @@
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F1" s="6" t="s">
         <v>3</v>
@@ -1232,7 +1232,7 @@
         <v>8</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>9</v>
@@ -1264,40 +1264,40 @@
         <v>2019</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>17</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H2" s="2">
         <v>248</v>
       </c>
       <c r="I2" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K2" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="N2" s="2" t="s">
+      <c r="O2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="P2" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>22</v>
       </c>
       <c r="Q2" s="2"/>
     </row>
@@ -1306,52 +1306,52 @@
         <v>14</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>24</v>
       </c>
       <c r="D3" s="2">
         <v>2018</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H3" s="2">
         <v>48</v>
       </c>
       <c r="I3" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="K3" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K3" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="O3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="Q3" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="Q3" s="2" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.2">
@@ -1359,49 +1359,49 @@
         <v>14</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="D4" s="2">
         <v>2017</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H4" s="2">
         <v>167</v>
       </c>
       <c r="I4" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="K4" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K4" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="N4" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="O4" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="Q4" s="2"/>
     </row>
@@ -1410,49 +1410,49 @@
         <v>14</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>34</v>
       </c>
       <c r="D5" s="2">
         <v>2017</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H5" s="2">
         <v>12</v>
       </c>
       <c r="I5" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="K5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K5" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="M5" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="N5" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="O5" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="Q5" s="2"/>
     </row>
@@ -1461,49 +1461,49 @@
         <v>14</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>38</v>
       </c>
       <c r="D6" s="2">
         <v>2013</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H6" s="2">
         <v>75</v>
       </c>
       <c r="I6" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="K6" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K6" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="M6" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="N6" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="O6" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="Q6" s="2"/>
     </row>
@@ -1512,52 +1512,52 @@
         <v>14</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>42</v>
       </c>
       <c r="D7" s="2">
         <v>2013</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H7" s="2">
         <v>121</v>
       </c>
       <c r="I7" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="K7" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K7" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="M7" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="N7" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="O7" s="2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P7" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q7" s="2" t="s">
         <v>44</v>
-      </c>
-      <c r="Q7" s="2" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
@@ -1565,52 +1565,52 @@
         <v>14</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>47</v>
       </c>
       <c r="D8" s="2">
         <v>2012</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H8" s="2">
         <v>20</v>
       </c>
       <c r="I8" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J8" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="K8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N8" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="O8" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="P8" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="Q8" s="2" t="s">
         <v>49</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="M8" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="N8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="O8" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="P8" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="Q8" s="2" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.2">
@@ -1618,52 +1618,52 @@
         <v>14</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>52</v>
       </c>
       <c r="D9" s="2">
         <v>2011</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H9" s="2">
         <v>95</v>
       </c>
       <c r="I9" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J9" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="K9" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K9" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="L9" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="M9" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="N9" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="O9" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="P9" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="Q9" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="P9" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="Q9" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.2">
@@ -1671,52 +1671,52 @@
         <v>14</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>57</v>
       </c>
       <c r="D10" s="2">
         <v>2008</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H10" s="2">
         <v>114</v>
       </c>
       <c r="I10" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J10" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="K10" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N10" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K10" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="L10" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="M10" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="N10" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="O10" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="P10" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.2">
@@ -1724,52 +1724,52 @@
         <v>14</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="D11" s="2">
         <v>2019</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H11" s="2">
         <v>100</v>
       </c>
       <c r="I11" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="K11" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N11" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K11" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="L11" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="M11" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="N11" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="O11" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P11" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="Q11" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.2">
@@ -1777,49 +1777,49 @@
         <v>14</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>65</v>
       </c>
       <c r="D12" s="2">
         <v>2008</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H12" s="2">
         <v>50</v>
       </c>
       <c r="I12" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J12" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J12" s="2" t="s">
+      <c r="K12" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="M12" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K12" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="L12" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="M12" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="N12" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="O12" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="P12" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="Q12" s="2"/>
     </row>
@@ -1828,49 +1828,49 @@
         <v>14</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>68</v>
       </c>
       <c r="D13" s="2">
         <v>2014</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H13" s="2">
         <v>16</v>
       </c>
       <c r="I13" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J13" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J13" s="2" t="s">
+      <c r="K13" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="M13" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K13" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="L13" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="M13" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="N13" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="O13" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P13" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="Q13" s="2"/>
     </row>
@@ -1879,49 +1879,49 @@
         <v>14</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>71</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>72</v>
       </c>
       <c r="D14" s="2">
         <v>2013</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H14" s="2">
         <v>6</v>
       </c>
       <c r="I14" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J14" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J14" s="2" t="s">
+      <c r="K14" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N14" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K14" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="L14" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="M14" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="N14" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="O14" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="P14" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="Q14" s="2"/>
     </row>
@@ -1930,49 +1930,49 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>76</v>
       </c>
       <c r="D15" s="2">
         <v>2015</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H15" s="2">
         <v>16</v>
       </c>
       <c r="I15" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J15" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J15" s="2" t="s">
+      <c r="K15" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N15" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K15" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="L15" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="M15" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="N15" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="O15" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="P15" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="Q15" s="2"/>
     </row>
@@ -1981,49 +1981,49 @@
         <v>14</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>79</v>
       </c>
       <c r="D16" s="2">
         <v>2015</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H16" s="2">
         <v>28</v>
       </c>
       <c r="I16" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J16" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J16" s="2" t="s">
+      <c r="K16" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N16" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K16" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="L16" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="M16" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="N16" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="O16" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="P16" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="Q16" s="2"/>
     </row>
@@ -2032,52 +2032,52 @@
         <v>14</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>82</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>83</v>
       </c>
       <c r="D17" s="2">
         <v>2018</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H17" s="2">
         <v>12</v>
       </c>
       <c r="I17" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J17" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J17" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="K17" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O17" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="P17" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="Q17" s="2" t="s">
         <v>85</v>
-      </c>
-      <c r="P17" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="Q17" s="2" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.2">
@@ -2085,52 +2085,52 @@
         <v>14</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>87</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>88</v>
       </c>
       <c r="D18" s="2">
         <v>2017</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H18" s="2">
         <v>45</v>
       </c>
       <c r="I18" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J18" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J18" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="K18" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N18" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="O18" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="P18" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="Q18" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="O18" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="P18" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="Q18" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.2">
@@ -2138,49 +2138,49 @@
         <v>14</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>93</v>
       </c>
       <c r="D19" s="2">
         <v>2017</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H19" s="2">
         <v>51</v>
       </c>
       <c r="I19" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J19" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J19" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="K19" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O19" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="P19" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="Q19" s="2"/>
     </row>
@@ -2189,52 +2189,52 @@
         <v>14</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>96</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>97</v>
       </c>
       <c r="D20" s="2">
         <v>2010</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H20" s="2">
         <v>16</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>18</v>
+        <v>227</v>
       </c>
       <c r="J20" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="M20" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="K20" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="L20" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="M20" s="2" t="s">
+      <c r="N20" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="N20" s="2" t="s">
+      <c r="O20" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="O20" s="2" t="s">
+      <c r="P20" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="Q20" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="P20" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="Q20" s="2" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.2">
@@ -2242,52 +2242,52 @@
         <v>14</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D21" s="2">
         <v>2017</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H21" s="2">
         <v>52</v>
       </c>
       <c r="I21" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J21" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J21" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="K21" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O21" s="2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="P21" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="Q21" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.2">
@@ -2295,49 +2295,49 @@
         <v>14</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>107</v>
       </c>
       <c r="D22" s="2">
         <v>2015</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H22" s="2">
         <v>35</v>
       </c>
       <c r="I22" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J22" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J22" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="K22" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O22" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="P22" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="Q22" s="2"/>
     </row>
@@ -2346,52 +2346,52 @@
         <v>14</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>110</v>
       </c>
       <c r="D23" s="2">
         <v>2009</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H23" s="2">
         <v>24</v>
       </c>
       <c r="I23" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J23" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J23" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="K23" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O23" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="P23" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="Q23" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.2">
@@ -2399,49 +2399,49 @@
         <v>14</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="D24" s="2">
         <v>2011</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H24" s="2">
         <v>66</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>18</v>
+        <v>227</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O24" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="P24" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="Q24" s="2"/>
     </row>
@@ -2450,52 +2450,52 @@
         <v>14</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>118</v>
       </c>
       <c r="D25" s="2">
         <v>2023</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H25" s="2">
         <v>24</v>
       </c>
       <c r="I25" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J25" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J25" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="K25" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L25" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O25" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="P25" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="Q25" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="P25" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="Q25" s="2" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.2">
@@ -2503,52 +2503,52 @@
         <v>14</v>
       </c>
       <c r="B26" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>123</v>
       </c>
       <c r="D26" s="2">
         <v>2022</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H26" s="2">
         <v>30</v>
       </c>
       <c r="I26" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J26" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J26" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="K26" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O26" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="P26" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="Q26" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.2">
@@ -2556,52 +2556,52 @@
         <v>14</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>130</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>131</v>
       </c>
       <c r="D27" s="2">
         <v>2021</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H27" s="2">
         <v>24</v>
       </c>
       <c r="I27" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J27" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J27" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="K27" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="M27" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N27" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O27" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="P27" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="Q27" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.2">
@@ -2609,52 +2609,52 @@
         <v>14</v>
       </c>
       <c r="B28" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>134</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>135</v>
       </c>
       <c r="D28" s="2">
         <v>2020</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H28" s="2">
         <v>17</v>
       </c>
       <c r="I28" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J28" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J28" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="K28" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L28" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="M28" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N28" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O28" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="P28" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="Q28" s="2" t="s">
         <v>137</v>
-      </c>
-      <c r="P28" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="Q28" s="2" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.2">
@@ -2662,52 +2662,52 @@
         <v>14</v>
       </c>
       <c r="B29" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>139</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>140</v>
       </c>
       <c r="D29" s="2">
         <v>2019</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H29" s="2">
         <v>20</v>
       </c>
       <c r="I29" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J29" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J29" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="K29" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L29" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="M29" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N29" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O29" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="P29" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="Q29" s="2" t="s">
         <v>142</v>
-      </c>
-      <c r="P29" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="Q29" s="2" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.2">
@@ -2715,52 +2715,52 @@
         <v>14</v>
       </c>
       <c r="B30" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>82</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>83</v>
       </c>
       <c r="D30" s="2">
         <v>2018</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H30" s="2">
         <v>12</v>
       </c>
       <c r="I30" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J30" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J30" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="K30" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="M30" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N30" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O30" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="P30" s="2" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="Q30" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.2">
@@ -2768,52 +2768,52 @@
         <v>14</v>
       </c>
       <c r="B31" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="D31" s="2">
         <v>2018</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H31" s="2">
         <v>24</v>
       </c>
       <c r="I31" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J31" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J31" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="K31" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="M31" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N31" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O31" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="P31" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="Q31" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.2">
@@ -2821,52 +2821,52 @@
         <v>14</v>
       </c>
       <c r="B32" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>149</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>150</v>
       </c>
       <c r="D32" s="2">
         <v>2018</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H32" s="2">
         <v>32</v>
       </c>
       <c r="I32" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J32" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J32" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="K32" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="M32" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O32" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="P32" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="Q32" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.2">
@@ -2874,52 +2874,52 @@
         <v>14</v>
       </c>
       <c r="B33" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>87</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>88</v>
       </c>
       <c r="D33" s="2">
         <v>2017</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H33" s="2">
         <v>43</v>
       </c>
       <c r="I33" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J33" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J33" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="K33" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N33" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O33" s="2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="P33" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="Q33" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.2">
@@ -2927,52 +2927,52 @@
         <v>14</v>
       </c>
       <c r="B34" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>155</v>
       </c>
       <c r="D34" s="2">
         <v>2015</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H34" s="2">
         <v>48</v>
       </c>
       <c r="I34" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J34" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J34" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="K34" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O34" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="P34" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="Q34" s="2" t="s">
         <v>157</v>
-      </c>
-      <c r="P34" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="Q34" s="2" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.2">
@@ -2980,52 +2980,52 @@
         <v>14</v>
       </c>
       <c r="B35" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C35" s="2" t="s">
         <v>159</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>160</v>
       </c>
       <c r="D35" s="2">
         <v>2018</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F35" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="G35" s="2" t="s">
         <v>161</v>
-      </c>
-      <c r="G35" s="2" t="s">
-        <v>162</v>
       </c>
       <c r="H35" s="2">
         <v>20</v>
       </c>
       <c r="I35" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J35" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J35" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="K35" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O35" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="P35" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="Q35" s="2" t="s">
         <v>163</v>
-      </c>
-      <c r="Q35" s="2" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.2">
@@ -3033,98 +3033,98 @@
         <v>14</v>
       </c>
       <c r="B36" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>126</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>127</v>
       </c>
       <c r="D36" s="2">
         <v>2021</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H36" s="2">
         <v>20</v>
       </c>
       <c r="I36" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J36" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J36" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="K36" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="M36" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O36" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="P36" s="5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="Q36" s="2"/>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B37" s="2"/>
       <c r="C37" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D37" s="2">
         <v>2025</v>
       </c>
       <c r="E37" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="F37" s="8" t="s">
         <v>221</v>
       </c>
-      <c r="F37" s="8" t="s">
-        <v>222</v>
-      </c>
       <c r="G37" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H37" s="2">
         <v>30</v>
       </c>
       <c r="I37" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K37" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="L37" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="M37" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N37" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="O37" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="J37" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K37" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="L37" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="M37" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="N37" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="O37" s="2" t="s">
+      <c r="P37" s="2" t="s">
         <v>224</v>
-      </c>
-      <c r="P37" s="2" t="s">
-        <v>225</v>
       </c>
       <c r="Q37" s="2"/>
     </row>

</xml_diff>